<commit_message>
updated GUI and Subscribers and interference py files
</commit_message>
<xml_diff>
--- a/logs/telegram_noc_bot_interactions.xlsx
+++ b/logs/telegram_noc_bot_interactions.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I273"/>
+  <dimension ref="A1:I317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="17.796875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -10597,13 +10597,11 @@
           <t>5928514077</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr"/>
       <c r="E273" t="inlineStr">
         <is>
           <t>Faraj saleh</t>
         </is>
       </c>
-      <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
           <t>5928514077</t>
@@ -10617,6 +10615,1636 @@
       <c r="I273" t="inlineStr">
         <is>
           <t>Disconnected sites with no power alarm: 9 - BGZ238 | Check TX/Link (No Power Alarm) | 2026-07-07 15:17:29 - COAST076 | Check TX/Link (No Power Alarm) | 2026-07-07 13:44:11 - COAST026 | Check TX/Link (No Power Alarm) | 2026-07-07 13:44:11 - COAST035 | Check TX/Link (No Power Alarm) | 2026-07-07 09:29:53 - BGZ139 | Check TX/Link (No Power Alarm) | 2026-07-04 13:19:43 - BGZ081 | Check TX/Link (No Power Alarm) | 2026-07-04 13:19:43 - BHZ015 | Check TX/Link (No Power Alarm) | 2026-06-01 09:56:17 - ECV001 | Check TX/Link (No Power Alarm) | 2026-05-20 10:11:47 - UECV001 | Check TX/Link (No Power A...</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-07-07 18:24:26</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-07-07 18:24:26</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-07-07_1820.xlsx Report snapshot: 2026-07-07 18:20 Report updated: 2026-07-07 18:20:34 Disconnected sites: 25 With power alarm: 15 No power alarm / check TX: 10 NetEco alarm rows: 61 MAE alarm rows: 25 Metrics from Excel: - Count of NE Is Disconnected: 25.0 - Count of Mains Failure: 61.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-07-07 18:24:28</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>search_site</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-07-07 18:24:28</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>Send the site name, for example ABZD001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-07-07 18:24:37</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>message_text</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Coast056</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-07-07 18:24:38</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>bot_reply</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Report: Final_NOC_Report_2026-07-07_1820.xlsx Site: COAST056 MO Name: COAST056 Alarm name: NE Is Disconnected MAE disconnect time: 2026-06-27 16:54:29 Power reason: Mains Failure Mains failure time: 2026-06-26 18:19:24 NetEco Current Alarms: - Minor | Mains Failure | 2026-06-26 18:19:24 MAE Current Alarms: - Critical | NE Is Disconnected | 2026-06-27 16:54:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-07-07 18:42:36</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-07-07 18:42:36</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-07-07_1840.xlsx Report snapshot: 2026-07-07 18:40 Report updated: 2026-07-07 18:40:35 Disconnected sites: 26 With power alarm: 16 No power alarm / check TX: 10 NetEco alarm rows: 52 MAE alarm rows: 26 Metrics from Excel: - Count of NE Is Disconnected: 26.0 - Count of Mains Failure: 52.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-07-07 18:42:42</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>nopower</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-07-07 18:42:43</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>Disconnected sites with no power alarm: 10 - JGBB001 | Check TX/Link (No Power Alarm) | 2026-07-07 17:55:47 - BGZ130 | Check TX/Link (No Power Alarm) | 2026-07-07 16:17:43 - BGZ129 | Check TX/Link (No Power Alarm) | 2026-07-07 16:17:43 - COAST076 | Check TX/Link (No Power Alarm) | 2026-07-07 13:44:11 - COAST026 | Check TX/Link (No Power Alarm) | 2026-07-07 13:44:11 - BGZ139 | Check TX/Link (No Power Alarm) | 2026-07-04 13:19:43 - BGZ081 | Check TX/Link (No Power Alarm) | 2026-07-04 13:19:43 - BHZ015 | Check TX/Link (No Power Alarm) | 2026-06-01 09:56:17 - ECV001 | Check TX/Link (No Power Al...</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-07-07 18:42:53</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>report</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-07-07 18:42:54</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>bot_sent_report</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Final_NOC_Report_2026-07-07_1840.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-07-07 19:55:08</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-07-07 19:55:11</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-07-07_1950.xlsx Report snapshot: 2026-07-07 19:50 Report updated: 2026-07-07 19:50:40 Disconnected sites: 24 With power alarm: 15 No power alarm / check TX: 9 NetEco alarm rows: 46 MAE alarm rows: 24 Metrics from Excel: - Count of NE Is Disconnected: 24.0 - Count of Mains Failure: 46.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-07-07 19:55:13</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-07-07 19:55:14</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-07-07_1950.xlsx Report snapshot: 2026-07-07 19:50 Report updated: 2026-07-07 19:50:40 Disconnected sites: 24 With power alarm: 15 No power alarm / check TX: 9 NetEco alarm rows: 46 MAE alarm rows: 24 Metrics from Excel: - Count of NE Is Disconnected: 24.0 - Count of Mains Failure: 46.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-07-07 19:55:16</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>search_site</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-07-07 19:55:16</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>Send the site name, for example ABZD001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-07-07 19:55:21</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>message_text</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-07-07 19:55:21</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>bot_reply</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Site '130' was not found in the latest report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-07-07 19:55:32</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>message_text</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>Bgz130</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-07-07 19:55:32</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>bot_reply</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>Site 'Bgz130' was not found in the latest report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-07-07 20:17:34</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>8693203957</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>هادي بالي</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>8693203957</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>nopower</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-07-07 20:17:35</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>8693203957</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>هادي بالي</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>8693203957</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>Disconnected sites with no power alarm: 7 - COAST076 | Check TX/Link (No Power Alarm) | 2026-07-07 13:44:11 - COAST026 | Check TX/Link (No Power Alarm) | 2026-07-07 13:44:11 - BGZ139 | Check TX/Link (No Power Alarm) | 2026-07-04 13:19:43 - BGZ081 | Check TX/Link (No Power Alarm) | 2026-07-04 13:19:43 - BHZ015 | Check TX/Link (No Power Alarm) | 2026-06-01 09:56:17 - ECV001 | Check TX/Link (No Power Alarm) | 2026-05-20 10:11:47 - UECV001 | Check TX/Link (No Power Alarm) | 2025-11-26 19:25:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-07-07 20:18:18</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>8693203957</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>هادي بالي</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>8693203957</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>neteco</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-07-07 20:18:18</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>8693203957</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>هادي بالي</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>8693203957</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>NetEco Current Alarms: 42 rows - SURT040 | Minor | Mains Failure | 2026-07-07 20:03:17 - DARN033 | Minor | Mains Failure | 2026-07-07 19:43:39 - DARN013 | Minor | Mains Failure | 2026-07-07 19:43:39 - DARN027 | Minor | Mains Failure | 2026-07-07 19:43:38 - DARN001 | Minor | Mains Failure | 2026-07-07 19:43:37 - MARJ013 | Minor | Mains Failure | 2026-07-07 19:41:54 - MARJ040 | Minor | Mains Failure | 2026-07-07 19:41:32 - BYDA025 | Minor | Mains Failure | 2026-07-07 19:32:34 - AGFT001 | Minor | Mains Failure | 2026-07-07 19:32:32 - BGZ045 | Minor | Mains Failure | 2026-07-07 19:03:30 - DARN0...</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-07-07 21:18:20</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>search_site</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-07-07 21:18:21</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>Send the site name, for example ABZD001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-07-07 21:18:33</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>message_text</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>Coast056</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-07-07 21:18:33</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>bot_reply</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>Report: Final_NOC_Report_2026-07-07_2115.xlsx Site: COAST056 MO Name: COAST056 Alarm name: NE Is Disconnected MAE disconnect time: 2026-06-27 16:54:29 Power reason: Mains Failure Mains failure time: 2026-06-26 18:19:24 NetEco Current Alarms: - Minor | Mains Failure | 2026-06-26 18:19:24 MAE Current Alarms: - Critical | NE Is Disconnected | 2026-06-27 16:54:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-07-07 21:19:00</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>search_site</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-07-07 21:19:01</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>Send the site name, for example ABZD001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-07-07 21:19:05</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>message_text</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>Bgz020</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-07-07 21:19:05</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>bot_reply</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>Report: Final_NOC_Report_2026-07-07_2115.xlsx Site: BGZ020 MO Name: BGZ020 Alarm name: NE Is Disconnected MAE disconnect time: 2026-07-02 00:36:31 Power reason: Mains Failure Mains failure time: 2026-07-03 14:39:31 NetEco Current Alarms: - Minor | Mains Failure | 2026-07-03 14:39:31 MAE Current Alarms: - Critical | NE Is Disconnected | 2026-07-02 00:36:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-07-07 21:59:19</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-07-07 21:59:20</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-07-07_2155.xlsx Report snapshot: 2026-07-07 21:55 Report updated: 2026-07-07 21:55:49 Disconnected sites: 16 With power alarm: 11 No power alarm / check TX: 5 NetEco alarm rows: 42 MAE alarm rows: 16 Metrics from Excel: - Count of NE Is Disconnected: 16.0 - Count of Mains Failure: 42.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-07-07 21:59:24</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>report</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-07-07 21:59:25</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>bot_sent_report</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>Final_NOC_Report_2026-07-07_2155.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-07-07 22:02:06</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>report</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-07-07 22:02:06</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>bot_sent_report</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>Final_NOC_Report_2026-07-07_2200.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-07-08 08:50:55</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-07-08 08:50:55</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-07-08_0846.xlsx Report snapshot: 2026-07-08 08:46 Report updated: 2026-07-08 08:46:11 Disconnected sites: 24 With power alarm: 0 No power alarm / check TX: 24 NetEco alarm rows: 0 MAE alarm rows: 24 Metrics from Excel: - Count of NE Is Disconnected: 24.0 - Count of Mains Failure: 0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-07-08 08:51:05</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-07-08 08:51:05</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr"/>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr"/>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-07-08_0846.xlsx Report snapshot: 2026-07-08 08:46 Report updated: 2026-07-08 08:46:11 Disconnected sites: 24 With power alarm: 0 No power alarm / check TX: 24 NetEco alarm rows: 0 MAE alarm rows: 24 Metrics from Excel: - Count of NE Is Disconnected: 24.0 - Count of Mains Failure: 0.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add orchestrator GUI, split scraper entry points, clean up legacy files
Introduces orchestrator_gui.py and standalone entry-point scripts for
each report (mae_scraper, neteco_scraper, ps_traffic_report,
subscriber_reports, merge_noc_reports), rewrites project_settings_gui.py
and telegram_noc_bot.py, and adds enhanced_noc_analysis.py,
neteco_dual_current_alarm_scraper.py, export_project_structure.py, a
README, .env.example, and a smoke test. Removes superseded/duplicate
scripts (copy all .py files.py, datacome.py, import Time.py,
subscribers_ftp_daily.py, subscribers_interference_monthly.py, user
complaint.py) and fixes requirements.txt to be UTF-8 instead of UTF-16.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/telegram_noc_bot_interactions.xlsx
+++ b/logs/telegram_noc_bot_interactions.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I323"/>
+  <dimension ref="A1:I417"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="17.796875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -12447,13 +12447,11 @@
           <t>5928514077</t>
         </is>
       </c>
-      <c r="D323" t="inlineStr"/>
       <c r="E323" t="inlineStr">
         <is>
           <t>Faraj saleh</t>
         </is>
       </c>
-      <c r="F323" t="inlineStr"/>
       <c r="G323" t="inlineStr">
         <is>
           <t>5928514077</t>
@@ -12467,6 +12465,3486 @@
       <c r="I323" t="inlineStr">
         <is>
           <t>NOC report: Final_NOC_Report_2026-07-09_0105.xlsx Report snapshot: 2026-07-09 01:05 Report updated: 2026-07-09 01:05:39 Disconnected sites: 25 With power alarm: 11 No power alarm / check TX: 14 NetEco alarm rows: 32 MAE alarm rows: 25 Metrics from Excel: - Count of NE Is Disconnected: 25.0 - Count of Mains Failure: 32.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-07-13 14:04:48</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>command_start</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>5104641346</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Walid</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>5104641346</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>/start</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-07-13 14:04:48</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>bot_reply</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>5104641346</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Walid</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>5104641346</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>Choose an option from the list, or type a site name directly. Examples: - ABZD001 - COAST073 - /alarm Mains Failure - /site BGZ162 - /phone</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-07-13 14:04:49</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>command_start</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>5104641346</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Walid</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>5104641346</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>/start</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-07-13 14:04:49</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>bot_reply</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>5104641346</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Walid</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>5104641346</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>Choose an option from the list, or type a site name directly. Examples: - ABZD001 - COAST073 - /alarm Mains Failure - /site BGZ162 - /phone</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:31:11</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:31:12</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-08-03_1126.xlsx Report snapshot: 2026-08-03 11:26 Report updated: 2026-08-03 11:26:43 Disconnected sites: 31 With power alarm: 22 No power alarm / check TX: 9 NetEco alarm rows: 94 MAE alarm rows: 31 Metrics from Excel: - Count of NE Is Disconnected: 31.0 - Count of Mains Failure: 94.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:32:24</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:32:24</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-08-03_1131.xlsx Report snapshot: 2026-08-03 11:31 Report updated: 2026-08-03 11:31:44 Disconnected sites: 34 With power alarm: 23 No power alarm / check TX: 11 NetEco alarm rows: 84 MAE alarm rows: 34 Metrics from Excel: - Count of NE Is Disconnected: 34.0 - Count of Mains Failure: 84.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:32:30</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>message_text</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>bgz070</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:32:31</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>bot_reply</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>Site 'bgz070' was not found in the latest report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:32:34</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>search_site</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:32:34</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>Send the site name, for example ABZD001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:32:37</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>message_text</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>bgz070</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:32:37</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>bot_reply</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>Site 'bgz070' was not found in the latest report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:35:35</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:35:35</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-08-03_1131.xlsx Report snapshot: 2026-08-03 11:31 Report updated: 2026-08-03 11:31:44 Disconnected sites: 34 With power alarm: 23 No power alarm / check TX: 11 NetEco alarm rows: 84 MAE alarm rows: 34 Metrics from Excel: - Count of NE Is Disconnected: 34.0 - Count of Mains Failure: 84.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:36:08</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:36:08</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-08-03_1131.xlsx Report snapshot: 2026-08-03 11:31 Report updated: 2026-08-03 11:31:44 Disconnected sites: 34 With power alarm: 23 No power alarm / check TX: 11 NetEco alarm rows: 84 MAE alarm rows: 34 Metrics from Excel: - Count of NE Is Disconnected: 34.0 - Count of Mains Failure: 84.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:36:10</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:36:10</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-08-03_1131.xlsx Report snapshot: 2026-08-03 11:31 Report updated: 2026-08-03 11:31:44 Disconnected sites: 34 With power alarm: 23 No power alarm / check TX: 11 NetEco alarm rows: 84 MAE alarm rows: 34 Metrics from Excel: - Count of NE Is Disconnected: 34.0 - Count of Mains Failure: 84.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:36:12</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>report</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-08-03 11:36:13</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>bot_sent_report</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>Final_NOC_Report_2026-08-03_1131.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-08-10 23:49:34</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-08-10 23:49:36</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-08-10_2346.xlsx Report snapshot: 2026-08-10 23:46 Report updated: 2026-08-10 23:46:13 Disconnected sites: 29 With power alarm: 17 No power alarm / check TX: 12 NetEco alarm rows: 53 MAE alarm rows: 29 Metrics from Excel: - Count of NE Is Disconnected: 29.0 - Count of Mains Failure: 53.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-08-10 23:49:39</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>search_site</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-08-10 23:49:40</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>Send the site name, for example ABZD001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-08-10 23:50:05</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>message_text</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>bgz165</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-08-10 23:50:05</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>bot_reply</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>Report: Final_NOC_Report_2026-08-10_2346.xlsx Site: BGZ165 MO Name: BGZ165(FN) Alarm name: NE Is Disconnected MAE disconnect time: 2026-08-10 21:55:03 Power reason: Mains Failure Mains failure time: 2026-08-10 21:26:12 NetEco Current Alarms: - Minor | Mains Failure | 2026-08-10 21:26:12 MAE Current Alarms: - Critical | NE Is Disconnected | 2026-08-10 21:55:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-08-10 23:50:15</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>report</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-08-10 23:50:16</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>bot_sent_report</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>Final_NOC_Report_2026-08-10_2346.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-08-11 00:06:12</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-08-11 00:06:13</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-08-10_2356.xlsx Report snapshot: 2026-08-10 23:56 Report updated: 2026-08-10 23:56:15 Disconnected sites: 30 With power alarm: 18 No power alarm / check TX: 12 NetEco alarm rows: 52 MAE alarm rows: 30 Metrics from Excel: - Count of NE Is Disconnected: 30.0 - Count of Mains Failure: 52.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:04:56</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:04:57</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-08-11_0901.xlsx Report snapshot: 2026-08-11 09:01 Report updated: 2026-08-11 09:01:38 Disconnected sites: 32 With power alarm: 17 No power alarm / check TX: 15 NetEco alarm rows: 50 MAE alarm rows: 32 Metrics from Excel: - Count of NE Is Disconnected: 32.0 - Count of Mains Failure: 50.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:05:01</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:05:01</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-08-11_0901.xlsx Report snapshot: 2026-08-11 09:01 Report updated: 2026-08-11 09:01:38 Disconnected sites: 32 With power alarm: 17 No power alarm / check TX: 15 NetEco alarm rows: 50 MAE alarm rows: 32 Metrics from Excel: - Count of NE Is Disconnected: 32.0 - Count of Mains Failure: 50.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:41:59</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:42:01</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-08-11_0941.xlsx Report snapshot: 2026-08-11 09:41 Report updated: 2026-08-11 09:41:44 Disconnected sites: 34 With power alarm: 19 No power alarm / check TX: 15 NetEco alarm rows: 50 MAE alarm rows: 34 Metrics from Excel: - Count of NE Is Disconnected: 34.0 - Count of Mains Failure: 50.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:42:07</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>report</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:42:08</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>bot_sent_report</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>Final_NOC_Report_2026-08-11_0941.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:49:03</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>Ahmed Muftah</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:49:04</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Ahmed Muftah</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-08-11_0946.xlsx Report snapshot: 2026-08-11 09:46 Report updated: 2026-08-11 09:46:44 Disconnected sites: 29 With power alarm: 19 No power alarm / check TX: 10 NetEco alarm rows: 50 MAE alarm rows: 29 Metrics from Excel: - Count of NE Is Disconnected: 29.0 - Count of Mains Failure: 50.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:49:09</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Ahmed Muftah</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>report</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:49:09</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>bot_sent_report</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Ahmed Muftah</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>Final_NOC_Report_2026-08-11_0946.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:50:12</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Ahmed Muftah</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>search_site</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:50:13</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Ahmed Muftah</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>Send the site name, for example ABZD001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:50:37</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>message_text</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>Ahmed Muftah</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>coast021</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:50:38</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>bot_reply</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Ahmed Muftah</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>8567160214</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>Report: Final_NOC_Report_2026-08-11_0946.xlsx Site: COAST021 MO Name: COAST021 Alarm name: NE Is Disconnected MAE disconnect time: 2026-08-11 09:06:47 Power reason: Mains Failure Mains failure time: 2026-08-10 23:04:39 NetEco Current Alarms: - Minor | Mains Failure | 2026-08-10 23:04:39 MAE Current Alarms: - Critical | NE Is Disconnected | 2026-08-11 09:06:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-08-11 10:52:31</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-08-11 10:52:32</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-08-11_1051.xlsx Report snapshot: 2026-08-11 10:51 Report updated: 2026-08-11 10:51:48 Disconnected sites: 30 With power alarm: 20 No power alarm / check TX: 10 NetEco alarm rows: 78 MAE alarm rows: 30 Metrics from Excel: - Count of NE Is Disconnected: 30.0 - Count of Mains Failure: 78.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-08-11 10:52:35</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>search_site</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-08-11 10:52:35</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>Send the site name, for example ABZD001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-08-11 10:52:43</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>message_text</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>Bgz001</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-08-11 10:52:43</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>bot_reply</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>Site 'Bgz001' was not found in the latest report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-08-11 10:52:58</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>message_text</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>Mesa001</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-08-11 10:52:58</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>bot_reply</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>Site 'Mesa001' was not found in the latest report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-08-11 10:53:07</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>message_text</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>Coast021</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-08-11 10:53:07</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>bot_reply</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>Report: Final_NOC_Report_2026-08-11_1051.xlsx Site: COAST021 MO Name: COAST021 Alarm name: NE Is Disconnected MAE disconnect time: 2026-08-11 09:06:47 Power reason: Mains Failure Mains failure time: 2026-08-10 23:04:39 NetEco Current Alarms: - Minor | Mains Failure | 2026-08-10 23:04:39 MAE Current Alarms: - Critical | NE Is Disconnected | 2026-08-11 09:06:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-08-11 10:54:00</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>disconnected</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-08-11 10:54:00</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>All disconnected sites: 30 - BGZ023 | Check TX/Link (No Power Alarm) | 2026-08-11 10:41:47 - BGZ159 | Mains Failure | 2026-08-11 10:36:13 - BGZ188 | Mains Failure | 2026-08-11 10:20:25 - COAST020 | Mains Failure | 2026-08-11 09:35:15 - COAST021 | Mains Failure | 2026-08-11 09:06:47 - BDIY001 | Mains Failure | 2026-08-11 07:46:43 - RBYN001 | Check TX/Link (No Power Alarm) | 2026-08-11 06:55:25 - TBRK038 | Mains Failure | 2026-08-11 06:16:57 - JADI001 | Mains Failure | 2026-08-11 04:54:43 - BGZ167 | Check TX/Link (No Power Alarm) | 2026-08-11 04:32:39 - BGZ131 | Check TX/Link (No Power Alarm)...</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-08-11 12:50:56</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-08-11 12:50:57</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>NOC report: Final_NOC_Report_2026-08-11_1246.xlsx Report snapshot: 2026-08-11 12:46 Report updated: 2026-08-11 12:46:53 Disconnected sites: 28 With power alarm: 17 No power alarm / check TX: 11 NetEco alarm rows: 79 MAE alarm rows: 28 Metrics from Excel: - Count of NE Is Disconnected: 28.0 - Count of Mains Failure: 79.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-08-11 12:59:44</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-08-11 12:59:45</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>Report updated: 2026-08-11 12:56:54 # of Disconnected sites: 30 With power alarm: 18 No power alarm / check TX: 12 NetEco alarm rows: 68 MAE alarm rows: 30 Metrics from Excel: - Count of NE Is Disconnected: 30.0 - Count of Mains Failure: 68.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:00:55</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:00:56</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>Report updated: 2026-08-11 12:56:54 =====================================NetEco alarm rows: 68 MAE alarm rows: 30 Metrics from Excel: - Count of NE Is Disconnected: 30.0 - Count of Mains Failure: 68.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:00:57</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:00:58</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>Report updated: 2026-08-11 12:56:54 =====================================NetEco alarm rows: 68 MAE alarm rows: 30 Metrics from Excel: - Count of NE Is Disconnected: 30.0 - Count of Mains Failure: 68.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:25</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:26</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>Report found, but summary sheet is empty: Final_NOC_Report_2026-08-11_1311.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:26</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>search_site</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:26</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>Send the site name, for example ABZD001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:26</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:26</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>Report found, but summary sheet is empty: Final_NOC_Report_2026-08-11_1311.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:26</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:27</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>Report found, but summary sheet is empty: Final_NOC_Report_2026-08-11_1311.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:27</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:27</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>Report found, but summary sheet is empty: Final_NOC_Report_2026-08-11_1311.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:53</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:53</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>Report found, but summary sheet is empty: Final_NOC_Report_2026-08-11_1311.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:55</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:55</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>Report found, but summary sheet is empty: Final_NOC_Report_2026-08-11_1311.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:56</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:56</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>Report found, but summary sheet is empty: Final_NOC_Report_2026-08-11_1311.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:56</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:56</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>Report found, but summary sheet is empty: Final_NOC_Report_2026-08-11_1311.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:57</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:16:57</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>Report found, but summary sheet is empty: Final_NOC_Report_2026-08-11_1311.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:18:55</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:18:55</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>Report updated: 2026-08-11 13:16:58 ===================================== NetEco alarm rows: 77 MAE alarm rows: 30 Metrics from Excel: - Count of NE Is Disconnected: 30.0 - Count of Mains Failure: 77.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:18:58</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:18:58</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>Report updated: 2026-08-11 13:16:58 ===================================== NetEco alarm rows: 77 MAE alarm rows: 30 Metrics from Excel: - Count of NE Is Disconnected: 30.0 - Count of Mains Failure: 77.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:19:00</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:19:01</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>bot_callback_reply</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr"/>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>Faraj saleh</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr"/>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>5928514077</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>private</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>Report updated: 2026-08-11 13:16:58 ===================================== NetEco alarm rows: 77 MAE alarm rows: 30 Metrics from Excel: - Count of NE Is Disconnected: 30.0 - Count of Mains Failure: 77.0</t>
         </is>
       </c>
     </row>

</xml_diff>